<commit_message>
Updates included: 1. Simplifying the table on index.qmd into an overview table 2. Creating an overview table for each dataset 3. Adding TASO case studies into callout boxes. 5. General formatting improvements
</commit_message>
<xml_diff>
--- a/administrative-database-guidance/data/tbl_equality_gaps_outcomes.xlsx
+++ b/administrative-database-guidance/data/tbl_equality_gaps_outcomes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MikaylaBoginsky\Documents\technicalguide\administrative-database-guidance\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED3402F2-99DF-4E22-80E4-14D61A2258E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60C6F7B3-6F5A-44F3-941E-8A6A78967724}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
   <si>
     <t>Outcome measure</t>
   </si>
@@ -34,12 +34,6 @@
     <t>Sample</t>
   </si>
   <si>
-    <t>Source</t>
-  </si>
-  <si>
-    <t>Primary: Earning</t>
-  </si>
-  <si>
     <t>Reported total PAYE UK earnings in relevant tax year, from the LEO dataset. This includes everyone with any PAYE earnings reported, and therefore will include both part-time and full-time employees.</t>
   </si>
   <si>
@@ -49,16 +43,10 @@
     <t>2002 and 2003 cohorts, at the time of collection nine years after KS4 2010/2011 and 2011/12</t>
   </si>
   <si>
-    <t>LEO dataset</t>
-  </si>
-  <si>
     <t>16 years after KS4 - corresponding to tax years 2017/2018 and 2018/2019 for the two cohorts respectively.</t>
   </si>
   <si>
     <t>2002 and 2003 cohorts, at time of collection corresponding to tax years 2017/2018 and 2018/19 for the two cohorts respectively</t>
-  </si>
-  <si>
-    <t>Primary: Employment status (9 and 15 years after KS4)</t>
   </si>
   <si>
     <t>Person recorded as being employed in the UK at any point in the relevant tax year, from the LEO dataset. This includes any record of employment, regardless of length or nature of employment.</t>
@@ -72,6 +60,18 @@
   </si>
   <si>
     <t>2002 and 2003 cohorts, at time of collection  corresponding to tax years 2017/2018 and 2018/19 for the two cohorts respectively</t>
+  </si>
+  <si>
+    <t>Primary: Earnings (9 years after KS4)</t>
+  </si>
+  <si>
+    <t>Primary: Earnings (16 years after KS4)</t>
+  </si>
+  <si>
+    <t>Primary: Employment status (9 years after KS4)</t>
+  </si>
+  <si>
+    <t>Primary: Employment status (16 years after KS4)</t>
   </si>
 </sst>
 </file>
@@ -122,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -133,9 +133,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -355,13 +352,15 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="B2:H6"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.6"/>
+  <dimension ref="B2:G6"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.5703125" customWidth="1"/>
+    <col min="4" max="4" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" ht="32" x14ac:dyDescent="0.75">
+    <row r="2" spans="2:7" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -374,87 +373,72 @@
       <c r="E2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+    </row>
+    <row r="3" spans="2:7" ht="153" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
+      <c r="D3" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
     </row>
-    <row r="3" spans="2:8" ht="153" customHeight="1" x14ac:dyDescent="0.95">
-      <c r="B3" s="1" t="s">
+    <row r="4" spans="2:7" ht="234" x14ac:dyDescent="0.35">
+      <c r="B4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+    </row>
+    <row r="5" spans="2:7" ht="153" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" s="5" t="s">
+      <c r="E5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+    </row>
+    <row r="6" spans="2:7" ht="144" x14ac:dyDescent="0.35">
+      <c r="B6" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-    </row>
-    <row r="4" spans="2:8" ht="323" x14ac:dyDescent="0.95">
-      <c r="B4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="3" t="s">
+      <c r="D6" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-    </row>
-    <row r="5" spans="2:8" ht="153" customHeight="1" x14ac:dyDescent="0.95">
-      <c r="B5" s="1" t="s">
+      <c r="E6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-    </row>
-    <row r="6" spans="2:8" ht="289" x14ac:dyDescent="0.95">
-      <c r="B6" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="F6" s="2"/>
       <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>